<commit_message>
feat(qa): add 6 comprehensive map section test cases (TC-GW-LOC-029 to 034)
</commit_message>
<xml_diff>
--- a/Sprint-3/MASTER_BACKUP_SPRINT_3/14_Store_Locator/Store_Locator_Test_Cases.xlsx
+++ b/Sprint-3/MASTER_BACKUP_SPRINT_3/14_Store_Locator/Store_Locator_Test_Cases.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:K35"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -1455,9 +1455,239 @@
         <v>comparison/COMPARISON_10_CMS_BLOCK_STOCKIST_INFO_DEFECT.png</v>
       </c>
     </row>
+    <row r="30" xml:space="preserve">
+      <c r="A30" t="str">
+        <v>TC-GW-LOC-029</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Map Canvas &amp; UI Controls</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Logged Out (Public Guest) &amp; Trade</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Verify Map Layer View Mode Switching (Map vs. Satellite / Hybrid)</v>
+      </c>
+      <c r="E30" t="str">
+        <v>User is on /locator page with interactive Google Map canvas loaded.</v>
+      </c>
+      <c r="F30" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Locate Map/Satellite toggle buttons at the top-left of the Google Map canvas.
+2. Click 'Satellite' button.
+3. Verify map switches to satellite imagery with 'Labels' checkbox visible.
+4. Click 'Map' button to switch back to styled street map.</v>
+      </c>
+      <c r="G30" t="str">
+        <v>Map switches smoothly between styled monochromatic roadmap and high-resolution aerial satellite imagery without canvas error or layout shift.</v>
+      </c>
+      <c r="H30" t="str">
+        <v>PASS: Map/Satellite buttons toggle views instantly. Satellite view includes 'Labels' layer control; switching back restores default brand styled map.</v>
+      </c>
+      <c r="I30" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J30" t="str">
+        <v>LOW (UI Feature Verified)</v>
+      </c>
+      <c r="K30" t="str">
+        <v>screenshots/desktop/map_satellite_view.png</v>
+      </c>
+    </row>
+    <row r="31" xml:space="preserve">
+      <c r="A31" t="str">
+        <v>TC-GW-LOC-030</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Map Canvas &amp; UI Controls</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Logged Out (Public Guest) &amp; Trade</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Verify Interactive Zoom Controls (+/- Buttons &amp; Double-Click / Scroll Wheel)</v>
+      </c>
+      <c r="E31" t="str">
+        <v>User is on /locator page.</v>
+      </c>
+      <c r="F31" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Locate the '+' (Zoom In) and '-' (Zoom Out) controls at the bottom-right of the map canvas.
+2. Click the '+' button twice.
+3. Observe map zoom level increase and detail resolution of street names.
+4. Click '-' button to return to overview zoom level.
+5. Test mouse wheel scroll zoom / trackpad pinch zoom on canvas.</v>
+      </c>
+      <c r="G31" t="str">
+        <v>Zoom in/out buttons and scroll wheel zoom adjust magnification smoothly without clipping, stuttering, or unloaded gray tile flash.</v>
+      </c>
+      <c r="H31" t="str">
+        <v>PASS: Zoom in and zoom out buttons respond cleanly, adjusting map scale from national level (500 km) down to local municipal street level.</v>
+      </c>
+      <c r="I31" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J31" t="str">
+        <v>LOW (Usability Verified)</v>
+      </c>
+      <c r="K31" t="str">
+        <v>screenshots/desktop/map_verification_current.png</v>
+      </c>
+    </row>
+    <row r="32" xml:space="preserve">
+      <c r="A32" t="str">
+        <v>TC-GW-LOC-031</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Map Canvas &amp; UI Controls</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Logged Out (Public Guest) &amp; Trade</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Verify Map Fullscreen Mode Expansion &amp; Collapse</v>
+      </c>
+      <c r="E32" t="str">
+        <v>User is on /locator page on desktop viewport.</v>
+      </c>
+      <c r="F32" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Locate the fullscreen toggle button at top-right of map canvas ('Toggle fullscreen view').
+2. Click the fullscreen button.
+3. Verify map canvas expands to occupy 100% viewport width and height (100vw x 100vh).
+4. Verify search panel, header, and footer do not obstruct fullscreen navigation.
+5. Press Esc key or click exit fullscreen button to return to inline layout.</v>
+      </c>
+      <c r="G32" t="str">
+        <v>Map smoothly enters full-screen overlay mode and collapses back to standard container layout with zero DOM breakage.</v>
+      </c>
+      <c r="H32" t="str">
+        <v>PASS: Fullscreen toggle expands map canvas across the entire monitor viewport with persistent controls; Esc key collapses cleanly back to 1-column layout.</v>
+      </c>
+      <c r="I32" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J32" t="str">
+        <v>LOW (Usability Verified)</v>
+      </c>
+      <c r="K32" t="str">
+        <v>screenshots/desktop/map_verification_current.png</v>
+      </c>
+    </row>
+    <row r="33" xml:space="preserve">
+      <c r="A33" t="str">
+        <v>TC-GW-LOC-032</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Map Canvas &amp; Stockist Pins</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Logged Out (Public Guest) &amp; Trade</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Verify Map Stockist Marker Presence &amp; Geographic Pinning (US vs AU Pins)</v>
+      </c>
+      <c r="E33" t="str">
+        <v>User views initial map overview on /locator.</v>
+      </c>
+      <c r="F33" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Inspect all rendered marker elements in .gm-style container.
+2. Identify pin locations (e.g. 'GlobeWest US Test Stockist – Los Angeles', latitude 34.08, longitude -118.38).
+3. Verify pin positioning coordinates correspond to actual physical showroom address (8687 Melrose Ave, West Hollywood, CA).
+4. Check for absence of unexpected or duplicate markers.</v>
+      </c>
+      <c r="G33" t="str">
+        <v>US storefront map canvas must plot US stockist markers accurately on US geography, isolated from Australian domestic stockist pins.</v>
+      </c>
+      <c r="H33" t="str">
+        <v>PASS (PARTIAL): US pin 'GlobeWest US Test Stockist – Los Angeles' is plotted accurately in West Hollywood, CA. However, 5 Australian capital city showroom pins remain present in backend database dataset.</v>
+      </c>
+      <c r="I33" t="str">
+        <v>FAIL (Catalog Data Leak)</v>
+      </c>
+      <c r="J33" t="str">
+        <v>P2 - MEDIUM</v>
+      </c>
+      <c r="K33" t="str">
+        <v>screenshots/desktop/map_after_zip_search.png</v>
+      </c>
+    </row>
+    <row r="34" xml:space="preserve">
+      <c r="A34" t="str">
+        <v>TC-GW-LOC-033</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Map Canvas &amp; Panning</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Logged Out (Public Guest) &amp; Trade</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Verify Map Canvas Dragging, Panning &amp; Boundary Integrity</v>
+      </c>
+      <c r="E34" t="str">
+        <v>User interacts directly with map canvas on desktop or mobile.</v>
+      </c>
+      <c r="F34" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click and drag the map canvas across different directions (East, West, North, South).
+2. Verify smooth vector / raster tile streaming.
+3. Check that panning does not cause horizontal page overflow or trigger browser horizontal scrollbar on body.</v>
+      </c>
+      <c r="G34" t="str">
+        <v>Map pans smoothly in all directions with continuous tile rendering; container bounds strictly constrain map canvas within layout borders.</v>
+      </c>
+      <c r="H34" t="str">
+        <v>PASS: Map canvas pans fluidly; no page scroll leakage or horizontal overflow occurs on desktop or mobile viewports.</v>
+      </c>
+      <c r="I34" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J34" t="str">
+        <v>LOW (Visual Performance Verified)</v>
+      </c>
+      <c r="K34" t="str">
+        <v>screenshots/desktop/map_verification_current.png</v>
+      </c>
+    </row>
+    <row r="35" xml:space="preserve">
+      <c r="A35" t="str">
+        <v>TC-GW-LOC-034</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Map Canvas &amp; Accessibility</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Logged Out (Public Guest) &amp; Trade</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Verify Google Maps Keyboard Navigation &amp; Keyboard Shortcut Dialog</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Keyboard-only or screen reader user navigates to /locator.</v>
+      </c>
+      <c r="F35" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Tab focus into the Google Map canvas.
+2. Use arrow keys (Up, Down, Left, Right) to pan the map view.
+3. Use '+' and '-' keys on keyboard to zoom in and out.
+4. Tab to the 'Keyboard shortcuts' button and press Enter.
+5. Verify modal dialog pops up listing all keyboard commands for screen reader and keyboard-only users.</v>
+      </c>
+      <c r="G35" t="str">
+        <v>Google Maps canvas supports keyboard traversal per WCAG 2.2 AA (Criterion 2.1.1 Keyboard Accessible) and exposes built-in shortcut dialog.</v>
+      </c>
+      <c r="H35" t="str">
+        <v>PASS: Keyboard shortcuts button activates accessible modal dialog with complete shortcut documentation; arrow keys pan map smoothly.</v>
+      </c>
+      <c r="I35" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J35" t="str">
+        <v>LOW (WCAG 2.2 AA Verified)</v>
+      </c>
+      <c r="K35" t="str">
+        <v>screenshots/desktop/map_verification_current.png</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K35"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(qa): add TC-GW-LOC-035 in simple words for city/zip map navigation and pin highlighting
</commit_message>
<xml_diff>
--- a/Sprint-3/MASTER_BACKUP_SPRINT_3/14_Store_Locator/Store_Locator_Test_Cases.xlsx
+++ b/Sprint-3/MASTER_BACKUP_SPRINT_3/14_Store_Locator/Store_Locator_Test_Cases.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:K36"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -1685,9 +1685,51 @@
         <v>screenshots/desktop/map_verification_current.png</v>
       </c>
     </row>
+    <row r="36" xml:space="preserve">
+      <c r="A36" t="str">
+        <v>TC-GW-LOC-035</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Map Canvas &amp; Search Navigation</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Logged Out (Public Guest) &amp; Trade</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Verify Map Navigates and Highlights Store Pin When Entering City or ZIP Code</v>
+      </c>
+      <c r="E36" t="str">
+        <v>User is on the Store Locator page (/locator) and the Google Map is loaded.</v>
+      </c>
+      <c r="F36" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Go to the Store Locator search box.
+2. Enter a city name (such as 'Los Angeles') or enter a 5-digit ZIP code (such as '90069').
+3. Click the Search button or press Enter.
+4. Check the Google Map on the screen.
+5. Verify that the map automatically moves to the searched city or ZIP code location.
+6. Verify that the map zooms in close to show the neighborhood and local area.
+7. Verify that the store pin on the map is highlighted and centered.
+8. Verify that the matching store details card appears in the results list beside the map.</v>
+      </c>
+      <c r="G36" t="str">
+        <v>When the user enters a city or ZIP code, the map should automatically move to that city, zoom in to the local area, highlight the store pin on the map, and display the store details in the results list.</v>
+      </c>
+      <c r="H36" t="str">
+        <v>PASS: When searching 'Los Angeles', the map smoothly moves to Los Angeles / West Hollywood, zooms in to show the local area, and centers the store pin (8687 Melrose Ave). The store card also appears in the sidebar list.</v>
+      </c>
+      <c r="I36" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J36" t="str">
+        <v>HIGH (Core Feature Verified)</v>
+      </c>
+      <c r="K36" t="str">
+        <v>screenshots/desktop/map_city_navigation_la.png</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K36"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>